<commit_message>
data update for 303
</commit_message>
<xml_diff>
--- a/TIMES-NZ/v303/BY_Trans.xlsx
+++ b/TIMES-NZ/v303/BY_Trans.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -683,7 +683,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>C_WSR-*-DirectH-GEO</t>
+          <t>C_*-HEATX-GEO</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>C*-NGA*</t>
+          <t>C*CK*-LPG*</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>C*-DSL*</t>
+          <t>C*CK*-NGA*</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -736,6 +736,182 @@
         </is>
       </c>
       <c r="D17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>NCAP_BND</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>C*SH-Boiler-LPG*</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>NCAP_BND</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>C*SH-Boiler-NGA*</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>NCAP_BND</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>C*WH*-NGA*</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>NCAP_BND</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>C*MPM-PET*</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>NCAP_BND</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>C*MPM-LPG*</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>NCAP_BND</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>C*MPM-NGA*</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>NCAP_BND</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>C*Boiler-DSL*</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>NCAP_BND</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>AFISH*-PET</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
         <is>
           <t>2</t>
         </is>

</xml_diff>